<commit_message>
Adapting to new gazebo world and trying to fix waypoint problem
</commit_message>
<xml_diff>
--- a/planilhas/coordenadas_visita.xlsx
+++ b/planilhas/coordenadas_visita.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="793">
   <si>
     <t xml:space="preserve">Model Name</t>
   </si>
@@ -2390,6 +2390,15 @@
   </si>
   <si>
     <t xml:space="preserve">ls_tpc6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ls_diversos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_svc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-41.765774</t>
   </si>
 </sst>
 </file>
@@ -2510,8 +2519,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D789"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D791"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.17"/>
   </cols>
@@ -13559,6 +13568,34 @@
         <v>-41.7657583333333</v>
       </c>
       <c r="D789" s="0" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="790" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A790" s="0" t="s">
+        <v>790</v>
+      </c>
+      <c r="B790" s="0" t="n">
+        <v>-3.123187</v>
+      </c>
+      <c r="C790" s="0" t="n">
+        <v>-41.765903</v>
+      </c>
+      <c r="D790" s="0" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="791" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A791" s="0" t="s">
+        <v>791</v>
+      </c>
+      <c r="B791" s="0" t="n">
+        <v>-3.122447</v>
+      </c>
+      <c r="C791" s="0" t="s">
+        <v>792</v>
+      </c>
+      <c r="D791" s="0" t="n">
         <v>77</v>
       </c>
     </row>

</xml_diff>